<commit_message>
Dodajanje vsebine in sprememba strukture
</commit_message>
<xml_diff>
--- a/Delovni listi/Rezultati-izpita-neizpolnjeno.xlsx
+++ b/Delovni listi/Rezultati-izpita-neizpolnjeno.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janka\OneDrive\Namizje\SŠ - MAT\Matematika-v-srednjem-strokovnem-izobrazevanju\Delovni listi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/27bd894ee34b290c/Namizje/SŠ - MAT/Matematika-v-srednjem-strokovnem-izobrazevanju/Delovni listi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{813E79BA-0FA6-4BF1-BBB0-3C1EBA7A4FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{5AE0828E-4573-4248-AF6F-B6C12D1E160B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5481957F-0242-471D-9EB8-DA3675392CF9}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-3405" windowWidth="29040" windowHeight="15720" xr2:uid="{9E657715-4B84-4354-8AB0-542D4006503C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9E657715-4B84-4354-8AB0-542D4006503C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Podatki" sheetId="1" r:id="rId1"/>
+    <sheet name="Končni dosežki" sheetId="2" r:id="rId1"/>
+    <sheet name="Podatki" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,6 +34,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -712,6 +735,1024 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="sl-SI"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="sl-SI"/>
+              <a:t>Končni</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="sl-SI" baseline="0"/>
+              <a:t> dosežki</a:t>
+            </a:r>
+            <a:endParaRPr lang="sl-SI"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="sl-SI"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-144D-4E7D-9B47-7D937D201165}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-144D-4E7D-9B47-7D937D201165}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-144D-4E7D-9B47-7D937D201165}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-144D-4E7D-9B47-7D937D201165}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-144D-4E7D-9B47-7D937D201165}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-144D-4E7D-9B47-7D937D201165}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-144D-4E7D-9B47-7D937D201165}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="sl-SI"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="bestFit"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Podatki!$X$11:$X$17</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>negativno</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>ni opravljal izpita</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Podatki!$Y$11:$Y$17</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000E-144D-4E7D-9B47-7D937D201165}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="bestFit"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="sl-SI"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="sl-SI"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{8B0F1034-79A1-4EE8-B4A2-2F21A3F8359E}">
+  <sheetPr/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="9297051" cy="6073205"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Grafikon 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{934D7572-F9DB-4789-04FC-EB5226974E3C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2598,10 +3639,15 @@
         <v>1</v>
       </c>
       <c r="X25" s="2"/>
-      <c r="Y25" s="2"/>
+      <c r="Y25" s="2">
+        <v>50</v>
+      </c>
       <c r="Z25" s="2"/>
       <c r="AA25" s="2"/>
-      <c r="AB25" s="2"/>
+      <c r="AB25" s="2" cm="1">
+        <f t="array" ref="AB25:AB29">FREQUENCY(N3:N117,Y25:Y28)</f>
+        <v>56</v>
+      </c>
       <c r="AC25" s="2">
         <v>1</v>
       </c>
@@ -2648,10 +3694,14 @@
         <v>2</v>
       </c>
       <c r="X26" s="2"/>
-      <c r="Y26" s="2"/>
+      <c r="Y26" s="2">
+        <v>63</v>
+      </c>
       <c r="Z26" s="2"/>
       <c r="AA26" s="2"/>
-      <c r="AB26" s="2"/>
+      <c r="AB26" s="2">
+        <v>11</v>
+      </c>
       <c r="AC26" s="2">
         <v>2</v>
       </c>
@@ -2716,10 +3766,14 @@
         <v>3</v>
       </c>
       <c r="X27" s="2"/>
-      <c r="Y27" s="2"/>
+      <c r="Y27" s="2">
+        <v>76</v>
+      </c>
       <c r="Z27" s="2"/>
       <c r="AA27" s="2"/>
-      <c r="AB27" s="2"/>
+      <c r="AB27" s="2">
+        <v>9</v>
+      </c>
       <c r="AC27" s="2">
         <v>3</v>
       </c>
@@ -2766,10 +3820,14 @@
         <v>4</v>
       </c>
       <c r="X28" s="2"/>
-      <c r="Y28" s="2"/>
+      <c r="Y28" s="2">
+        <v>89</v>
+      </c>
       <c r="Z28" s="2"/>
       <c r="AA28" s="2"/>
-      <c r="AB28" s="2"/>
+      <c r="AB28" s="2">
+        <v>1</v>
+      </c>
       <c r="AC28" s="2">
         <v>4</v>
       </c>
@@ -2836,10 +3894,14 @@
         <v>5</v>
       </c>
       <c r="X29" s="2"/>
-      <c r="Y29" s="2"/>
+      <c r="Y29" s="2">
+        <v>100</v>
+      </c>
       <c r="Z29" s="2"/>
       <c r="AA29" s="2"/>
-      <c r="AB29" s="2"/>
+      <c r="AB29" s="2">
+        <v>2</v>
+      </c>
       <c r="AC29" s="2">
         <v>5</v>
       </c>
@@ -2903,7 +3965,7 @@
       </c>
       <c r="AB30" s="9">
         <f>SUM(AB25:AB29)</f>
-        <v>0</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:29" x14ac:dyDescent="0.25">

</xml_diff>